<commit_message>
Implement auth rollback, logout-home UX, docs/manual updates, and test tooling
</commit_message>
<xml_diff>
--- a/Call_Assignments/call_assignments.xlsx
+++ b/Call_Assignments/call_assignments.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -933,6 +933,1181 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Surayatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>[Boateng, Michael]_312-+302786248_20250923124023(2757).wav</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Boateng, Michael</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Boateng, Michael]_312-+302786248_20250923124023(2757).wav</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-08-03 09:32:16</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Surayatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>[Otchere, Ruth]_301-+233541906754_20250926134807(4439).wav</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Otchere, Ruth</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Otchere, Ruth]_301-+233541906754_20250926134807(4439).wav</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-08-03 09:32:16</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Surayatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>[Ewusie Moses, Anna]_310-+233240534802_20250924112631(3245).wav</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ewusie Moses, Anna</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Ewusie Moses, Anna]_310-+233240534802_20250924112631(3245).wav</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-08-03 09:32:16</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Surayatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>[Bortey, William]_305-+233596240003_20250923131915(2810).wav</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Bortey, William</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Bortey, William]_305-+233596240003_20250923131915(2810).wav</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-08-03 09:32:16</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Surayatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>[Boateng, Michael]_312-+233547338910_20250930162835(852).wav</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Boateng, Michael</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Boateng, Michael]_312-+233547338910_20250930162835(852).wav</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-08-03 09:32:16</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Araba Quartey</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>araba.quartey@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>[Ewusie Moses, Anna]_310-+233559103134_20250926145115(4510).wav</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Ewusie Moses, Anna</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Ewusie Moses, Anna]_310-+233559103134_20250926145115(4510).wav</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:36:22</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Araba Quartey</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>araba.quartey@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>[Otchere, Ruth]_301-+233546082840_20250925115812(3812).wav</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Otchere, Ruth</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Otchere, Ruth]_301-+233546082840_20250925115812(3812).wav</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:36:22</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Araba Quartey</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>araba.quartey@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>[Oku, Daina]_306-+233201793160_20250929110546(198).wav</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Oku, Daina</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Oku, Daina]_306-+233201793160_20250929110546(198).wav</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:36:22</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Araba Quartey</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>araba.quartey@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>[Tagoe, Ellis]_303-+233244304956_20250925103830(3701).wav</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Tagoe, Ellis</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Tagoe, Ellis]_303-+233244304956_20250925103830(3701).wav</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:36:22</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Araba Quartey</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>araba.quartey@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>[Tagoe, Ellis]_303-+233559689482_20250923123726(2756).wav</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Tagoe, Ellis</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Tagoe, Ellis]_303-+233559689482_20250923123726(2756).wav</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:36:22</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Surayatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>[Boateng, Michael]_312-+302739361_20250924182646(3547).wav</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Boateng, Michael</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Boateng, Michael]_312-+302739361_20250924182646(3547).wav</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:36:22</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Surayatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>[Atsu, Bennet]_304-+233547450156_20250924155632(3468) (1).wav</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Atsu, Bennet</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Atsu, Bennet]_304-+233547450156_20250924155632(3468) (1).wav</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:36:22</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Surayatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>[Bortey, William]_305-+233556615663_20250926081848(4102).wav</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Bortey, William</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Bortey, William]_305-+233556615663_20250926081848(4102).wav</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:36:22</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Surayatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>[Awinbilla, Linda]_311-+233546331005_20250929092613(125).wav</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Awinbilla, Linda</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Awinbilla, Linda]_311-+233546331005_20250929092613(125).wav</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:36:22</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Surayatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>[Oku, Daina]_306-+233203885735_20250923100210(2670).wav</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Oku, Daina</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Documents\python_projects\QA call audit tool\New call list\[Oku, Daina]_306-+233203885735_20250923100210(2670).wav</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:36:22</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Araba Quartey</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>araba.quartey@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>[Bortey, William]_305-+233247487125_20251017085718(1729).wav</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Bortey, William</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Desktop\Desktop\ACTUARIAL\QA\recorded calls\[Bortey, William]_305-+233247487125_20251017085718(1729).wav</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:40:53</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Araba Quartey</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>araba.quartey@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>[Boateng, Michael]_312-+233244570938_20251016125835(1400).wav</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Boateng, Michael</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Desktop\Desktop\ACTUARIAL\QA\recorded calls\[Boateng, Michael]_312-+233244570938_20251016125835(1400).wav</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:40:53</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Araba Quartey</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>araba.quartey@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>[Tagoe, Ellis]_303-+233248580792_20251001111834(1035).wav</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Tagoe, Ellis</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Desktop\Desktop\ACTUARIAL\QA\recorded calls\[Tagoe, Ellis]_303-+233248580792_20251001111834(1035).wav</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:40:53</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Araba Quartey</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>araba.quartey@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>[Boateng, Michael]_312-+233543287008_20251016133021(1414).wav</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Boateng, Michael</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Desktop\Desktop\ACTUARIAL\QA\recorded calls\[Boateng, Michael]_312-+233543287008_20251016133021(1414).wav</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:40:53</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Araba Quartey</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>araba.quartey@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>[Oku, Daina]_306-+233558746940_20251014150638(457).wav</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Oku, Daina</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Desktop\Desktop\ACTUARIAL\QA\recorded calls\[Oku, Daina]_306-+233558746940_20251014150638(457).wav</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:40:53</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Suraiyatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>[Boateng, Michael]_312-+233556450151_20251016133725(1416).wav</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Boateng, Michael</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Desktop\Desktop\ACTUARIAL\QA\recorded calls\[Boateng, Michael]_312-+233556450151_20251016133725(1416).wav</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:40:53</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Suraiyatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>[Atsu, Bennet]_304-+233244484582_20251014121347(305).wav</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Atsu, Bennet</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Desktop\Desktop\ACTUARIAL\QA\recorded calls\[Atsu, Bennet]_304-+233244484582_20251014121347(305).wav</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:40:53</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Suraiyatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>[Atsu, Bennet]_304-+233247643893_20251014172629(632).wav</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Atsu, Bennet</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Desktop\Desktop\ACTUARIAL\QA\recorded calls\[Atsu, Bennet]_304-+233247643893_20251014172629(632).wav</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:40:53</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Suraiyatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>[Atsu, Bennet]_304-+233246338545_20251014121207(301).wav</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Atsu, Bennet</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Desktop\Desktop\ACTUARIAL\QA\recorded calls\[Atsu, Bennet]_304-+233246338545_20251014121207(301).wav</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:40:53</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Suraiyatu Mohammed</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>suraiyatu.mohammed@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>[Oku, Daina]_306-+233243770108_20251014170309(621).wav</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Oku, Daina</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>C:\Users\a.biomarfo\OneDrive - Nationwide Medical Insurance\Desktop\Desktop\ACTUARIAL\QA\recorded calls\[Oku, Daina]_306-+233243770108_20251014170309(621).wav</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Edem Dzitrie</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>edem.dzitrie@nationwidemh.com</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2026-08-03 16:40:53</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>